<commit_message>
Update test results & matlab runners
</commit_message>
<xml_diff>
--- a/results/comparison_outputs_global_models_.xlsx
+++ b/results/comparison_outputs_global_models_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jason\OneDrive\Desktop\Research\UBC\ProjectKickoff\ATC138Comparison_tests_\comparison_scripts_post_release\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{589F2A53-AAB5-44B6-BFCC-AFA122C2EA69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D59E9EC-BCCF-472E-8DF8-F528B4132F46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9F5F1FA4-9B25-4F82-8B27-64E924962748}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
   <si>
     <t>model</t>
   </si>
@@ -204,6 +204,75 @@
   </si>
   <si>
     <t>haseltonRCMF_4story_batch</t>
+  </si>
+  <si>
+    <t>1927_W1a_2_IM1</t>
+  </si>
+  <si>
+    <t>1927_W1a_2_IM2</t>
+  </si>
+  <si>
+    <t>1927_W1a_2_IM3</t>
+  </si>
+  <si>
+    <t>1927_W1a_2_IM4</t>
+  </si>
+  <si>
+    <t>1927_W1a_2_IM5</t>
+  </si>
+  <si>
+    <t>1967_W2b_3_IM1</t>
+  </si>
+  <si>
+    <t>1967_W2b_3_IM2</t>
+  </si>
+  <si>
+    <t>1967_W2b_3_IM3</t>
+  </si>
+  <si>
+    <t>1967_W2b_3_IM4</t>
+  </si>
+  <si>
+    <t>1967_W2b_3_IM5</t>
+  </si>
+  <si>
+    <t>1985_W1a_1_IM2</t>
+  </si>
+  <si>
+    <t>1985_W1a_1_IM3</t>
+  </si>
+  <si>
+    <t>1985_W1a_1_IM4</t>
+  </si>
+  <si>
+    <t>1985_W1a_1_IM5</t>
+  </si>
+  <si>
+    <t>1985_W1a_2_IM1</t>
+  </si>
+  <si>
+    <t>1985_W1a_2_IM2</t>
+  </si>
+  <si>
+    <t>1985_W1a_2_IM3</t>
+  </si>
+  <si>
+    <t>1985_W1a_2_IM4</t>
+  </si>
+  <si>
+    <t>1985_W1a_2_IM5</t>
+  </si>
+  <si>
+    <t>1985_W1a_2_IM6</t>
+  </si>
+  <si>
+    <t>1985_W1a_2_IM7</t>
+  </si>
+  <si>
+    <t>1985_W1a_2_IM8</t>
+  </si>
+  <si>
+    <t>Models with missing SP3 components</t>
   </si>
 </sst>
 </file>
@@ -349,7 +418,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -529,8 +598,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="18">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -725,6 +800,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -770,7 +860,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
@@ -784,8 +874,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -869,6 +964,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFFCC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -892,7 +992,7 @@
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1122,13 +1222,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1880,11 +1980,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F93FED4-3570-48B5-B751-6F8E95F5C203}">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" customWidth="1"/>
     <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
@@ -1893,6 +1993,7 @@
     <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6" customWidth="1"/>
+    <col min="11" max="11" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1956,25 +2057,25 @@
       <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="13">
         <v>1.2073333333347499E-2</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="13">
         <v>1.24074209257432E-2</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="13">
         <v>1.6273224043715799E-3</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="13">
         <v>6.6687500000000201E-3</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="14">
         <v>97.307356666666607</v>
       </c>
-      <c r="H4" t="b">
+      <c r="H4" s="12" t="b">
         <f>AND(C4&gt;$C$1, D4&gt;$D$1)</f>
         <v>0</v>
       </c>
@@ -1987,30 +2088,30 @@
       <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="13">
         <v>1.3801849206349399</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="13">
         <v>1.00788029551631</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="13">
         <v>3.9966530054644797E-3</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="13">
         <v>1.392E-2</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="14">
         <v>136.93936936507899</v>
       </c>
-      <c r="H5" t="b">
-        <f t="shared" ref="H5:H43" si="0">AND(C5&gt;$C$1, D5&gt;$D$1)</f>
+      <c r="H5" s="12" t="b">
+        <f t="shared" ref="H5:H68" si="0">AND(C5&gt;$C$1, D5&gt;$D$1)</f>
         <v>0</v>
       </c>
       <c r="I5" s="5" t="b">
-        <f t="shared" ref="I5:I43" si="1">AND(F5&gt;$F$1,E5&gt;$E$1)</f>
+        <f t="shared" ref="I5:I68" si="1">AND(F5&gt;$F$1,E5&gt;$E$1)</f>
         <v>0</v>
       </c>
     </row>
@@ -2018,25 +2119,25 @@
       <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="13">
         <v>0.61887174603177098</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="13">
         <v>0.31880342641132198</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="13">
         <v>5.4982915813016004E-3</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="13">
         <v>1.51698348497944E-2</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="14">
         <v>194.12330444444399</v>
       </c>
-      <c r="H6" t="b">
+      <c r="H6" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2049,25 +2150,25 @@
       <c r="A7" s="4">
         <v>4</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="13">
         <v>0.50209746031754299</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="13">
         <v>0.14967439945820299</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="13">
         <v>7.64894765077225E-3</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="13">
         <v>2.1044889836835001E-2</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="14">
         <v>335.45981285714203</v>
       </c>
-      <c r="H7" t="b">
+      <c r="H7" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2080,25 +2181,25 @@
       <c r="A8" s="4">
         <v>5</v>
       </c>
-      <c r="B8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="11">
-        <v>1.07999999999999E-2</v>
-      </c>
-      <c r="D8" s="11">
-        <v>2.6137463697966998</v>
-      </c>
-      <c r="E8" s="11">
-        <v>4.5355191256830498E-5</v>
-      </c>
-      <c r="F8" s="11">
-        <v>1.7333333333333301E-4</v>
-      </c>
-      <c r="G8" s="11">
-        <v>0.41320000000000001</v>
-      </c>
-      <c r="H8" t="b">
+      <c r="B8" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="13">
+        <v>1.54E-2</v>
+      </c>
+      <c r="D8" s="13">
+        <v>0.86546026750590499</v>
+      </c>
+      <c r="E8" s="13">
+        <v>2.1995416887008601E-4</v>
+      </c>
+      <c r="F8" s="13">
+        <v>8.0937499999999998E-4</v>
+      </c>
+      <c r="G8" s="14">
+        <v>1.7794000000000001</v>
+      </c>
+      <c r="H8" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2111,25 +2212,25 @@
       <c r="A9" s="4">
         <v>6</v>
       </c>
-      <c r="B9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="11">
-        <v>4.7400000000000497E-2</v>
-      </c>
-      <c r="D9" s="11">
-        <v>1.0119267883066301</v>
-      </c>
-      <c r="E9" s="11">
-        <v>3.6147540983606601E-4</v>
-      </c>
-      <c r="F9" s="11">
-        <v>1.54999999999999E-3</v>
-      </c>
-      <c r="G9" s="11">
-        <v>4.6841333333333299</v>
-      </c>
-      <c r="H9" t="b">
+      <c r="B9" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="13">
+        <v>0.24439999999999801</v>
+      </c>
+      <c r="D9" s="13">
+        <v>0.76448103498970499</v>
+      </c>
+      <c r="E9" s="13">
+        <v>1.84644808743169E-3</v>
+      </c>
+      <c r="F9" s="13">
+        <v>9.7633333333333391E-3</v>
+      </c>
+      <c r="G9" s="14">
+        <v>31.9694</v>
+      </c>
+      <c r="H9" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2142,25 +2243,25 @@
       <c r="A10" s="4">
         <v>7</v>
       </c>
-      <c r="B10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="11">
-        <v>6.7000000000000101E-2</v>
-      </c>
-      <c r="D10" s="11">
-        <v>0.34428301776911502</v>
-      </c>
-      <c r="E10" s="11">
-        <v>9.89344262295082E-4</v>
-      </c>
-      <c r="F10" s="11">
-        <v>3.3333333333333301E-3</v>
-      </c>
-      <c r="G10" s="11">
-        <v>19.460733333333302</v>
-      </c>
-      <c r="H10" t="b">
+      <c r="B10" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="13">
+        <v>1.0602</v>
+      </c>
+      <c r="D10" s="13">
+        <v>1.68974486478216</v>
+      </c>
+      <c r="E10" s="13">
+        <v>2.91398907103825E-3</v>
+      </c>
+      <c r="F10" s="13">
+        <v>1.37466666666666E-2</v>
+      </c>
+      <c r="G10" s="14">
+        <v>62.743200000000002</v>
+      </c>
+      <c r="H10" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2173,25 +2274,25 @@
       <c r="A11" s="4">
         <v>8</v>
       </c>
-      <c r="B11" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="11">
-        <v>0.61400000000000399</v>
-      </c>
-      <c r="D11" s="11">
-        <v>1.1527471303355299</v>
-      </c>
-      <c r="E11" s="11">
-        <v>1.65543803983783E-3</v>
-      </c>
-      <c r="F11" s="11">
-        <v>7.4349999999999998E-3</v>
-      </c>
-      <c r="G11" s="11">
-        <v>53.264066666666601</v>
-      </c>
-      <c r="H11" t="b">
+      <c r="B11" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="13">
+        <v>0.183199999999999</v>
+      </c>
+      <c r="D11" s="13">
+        <v>0.23566580736121101</v>
+      </c>
+      <c r="E11" s="13">
+        <v>3.1291803278688502E-3</v>
+      </c>
+      <c r="F11" s="13">
+        <v>9.7183333333333705E-3</v>
+      </c>
+      <c r="G11" s="14">
+        <v>77.737200000000001</v>
+      </c>
+      <c r="H11" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2204,25 +2305,25 @@
       <c r="A12" s="4">
         <v>9</v>
       </c>
-      <c r="B12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="11">
-        <v>9.1799999999985005E-2</v>
-      </c>
-      <c r="D12" s="11">
-        <v>0.170463196909104</v>
-      </c>
-      <c r="E12" s="11">
-        <v>2.2864216463951998E-3</v>
-      </c>
-      <c r="F12" s="11">
-        <v>1.005E-2</v>
-      </c>
-      <c r="G12" s="11">
-        <v>53.853266666666599</v>
-      </c>
-      <c r="H12" t="b">
+      <c r="B12" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="13">
+        <v>0.113799999999997</v>
+      </c>
+      <c r="D12" s="13">
+        <v>0.116892027922606</v>
+      </c>
+      <c r="E12" s="13">
+        <v>3.12379954563308E-3</v>
+      </c>
+      <c r="F12" s="13">
+        <v>1.6452293453110101E-2</v>
+      </c>
+      <c r="G12" s="14">
+        <v>97.354799999999997</v>
+      </c>
+      <c r="H12" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2235,25 +2336,25 @@
       <c r="A13" s="4">
         <v>10</v>
       </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="11">
-        <v>0.33222666666667</v>
-      </c>
-      <c r="D13" s="11">
-        <v>0.38132982032880602</v>
-      </c>
-      <c r="E13" s="11">
-        <v>2.4495129484438001E-3</v>
-      </c>
-      <c r="F13" s="11">
-        <v>8.1496461071789393E-3</v>
-      </c>
-      <c r="G13" s="11">
-        <v>87.123180238095202</v>
-      </c>
-      <c r="H13" t="b">
+      <c r="B13" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="13">
+        <v>0.16339999999999899</v>
+      </c>
+      <c r="D13" s="13">
+        <v>14.0837786588519</v>
+      </c>
+      <c r="E13" s="13">
+        <v>4.3489335448616199E-4</v>
+      </c>
+      <c r="F13" s="13">
+        <v>1.55499999999999E-3</v>
+      </c>
+      <c r="G13" s="14">
+        <v>1.1601999999999999</v>
+      </c>
+      <c r="H13" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2266,25 +2367,25 @@
       <c r="A14" s="4">
         <v>11</v>
       </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="11">
-        <v>0.94603166666666905</v>
-      </c>
-      <c r="D14" s="11">
-        <v>0.98245718857136299</v>
-      </c>
-      <c r="E14" s="11">
-        <v>2.3826473488076701E-3</v>
-      </c>
-      <c r="F14" s="11">
-        <v>9.5786612300372796E-3</v>
-      </c>
-      <c r="G14" s="11">
-        <v>96.2924061904762</v>
-      </c>
-      <c r="H14" t="b">
+      <c r="B14" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="13">
+        <v>4.6833333333466901E-3</v>
+      </c>
+      <c r="D14" s="13">
+        <v>6.8264012160420299E-3</v>
+      </c>
+      <c r="E14" s="13">
+        <v>1.2174863387978099E-3</v>
+      </c>
+      <c r="F14" s="13">
+        <v>5.8316666666666699E-3</v>
+      </c>
+      <c r="G14" s="14">
+        <v>68.606183333333306</v>
+      </c>
+      <c r="H14" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2297,25 +2398,25 @@
       <c r="A15" s="4">
         <v>12</v>
       </c>
-      <c r="B15" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="11">
-        <v>2.5457857142867999E-2</v>
-      </c>
-      <c r="D15" s="11">
-        <v>1.8492558662752699E-2</v>
-      </c>
-      <c r="E15" s="11">
-        <v>2.8569606841097198E-3</v>
-      </c>
-      <c r="F15" s="11">
-        <v>9.4118676089846101E-3</v>
-      </c>
-      <c r="G15" s="11">
-        <v>137.66541238095201</v>
-      </c>
-      <c r="H15" t="b">
+      <c r="B15" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="13">
+        <v>0.55893333333334205</v>
+      </c>
+      <c r="D15" s="13">
+        <v>0.64120679033709105</v>
+      </c>
+      <c r="E15" s="13">
+        <v>2.9086338797814199E-3</v>
+      </c>
+      <c r="F15" s="13">
+        <v>1.44716666666667E-2</v>
+      </c>
+      <c r="G15" s="14">
+        <v>87.168966666666606</v>
+      </c>
+      <c r="H15" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2328,25 +2429,25 @@
       <c r="A16" s="4">
         <v>13</v>
       </c>
-      <c r="B16" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="11">
-        <v>0</v>
-      </c>
-      <c r="D16" s="11">
-        <v>0</v>
-      </c>
-      <c r="E16" s="11">
-        <v>0</v>
-      </c>
-      <c r="F16" s="11">
-        <v>0</v>
-      </c>
-      <c r="G16" s="11">
-        <v>0</v>
-      </c>
-      <c r="H16" t="b">
+      <c r="B16" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="13">
+        <v>0.19633333333334199</v>
+      </c>
+      <c r="D16" s="13">
+        <v>0.13876579020403601</v>
+      </c>
+      <c r="E16" s="13">
+        <v>3.3809500763175098E-3</v>
+      </c>
+      <c r="F16" s="13">
+        <v>1.6260162601626001E-2</v>
+      </c>
+      <c r="G16" s="14">
+        <v>141.4854</v>
+      </c>
+      <c r="H16" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2355,29 +2456,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>14</v>
       </c>
-      <c r="B17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="11">
-        <v>7.5600000000000001E-2</v>
-      </c>
-      <c r="D17" s="11">
-        <v>13.705583756345099</v>
-      </c>
-      <c r="E17" s="11">
-        <v>1.15300546448087E-4</v>
-      </c>
-      <c r="F17" s="11">
-        <v>4.4999999999999999E-4</v>
-      </c>
-      <c r="G17" s="11">
-        <v>0.55159999999999998</v>
-      </c>
-      <c r="H17" t="b">
+      <c r="B17" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="13">
+        <v>6.2866666666650403E-2</v>
+      </c>
+      <c r="D17" s="13">
+        <v>1.6919808897661998E-2</v>
+      </c>
+      <c r="E17" s="13">
+        <v>1.1984810595535699E-2</v>
+      </c>
+      <c r="F17" s="13">
+        <v>3.8954802259886998E-2</v>
+      </c>
+      <c r="G17" s="14">
+        <v>371.5566</v>
+      </c>
+      <c r="H17" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2386,29 +2487,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>15</v>
       </c>
-      <c r="B18" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18" s="11">
-        <v>2.6599999999999201E-2</v>
-      </c>
-      <c r="D18" s="11">
-        <v>0.56101573374950997</v>
-      </c>
-      <c r="E18" s="11">
-        <v>3.72404371584699E-4</v>
-      </c>
-      <c r="F18" s="11">
-        <v>1.5149999999999901E-3</v>
-      </c>
-      <c r="G18" s="11">
-        <v>4.7413999999999996</v>
-      </c>
-      <c r="H18" t="b">
+      <c r="B18" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="13">
+        <v>3.0599999999999999E-2</v>
+      </c>
+      <c r="D18" s="13">
+        <v>11.103047895500699</v>
+      </c>
+      <c r="E18" s="13">
+        <v>1.13661202185792E-4</v>
+      </c>
+      <c r="F18" s="13">
+        <v>5.2564516129032196E-4</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0.27560000000000001</v>
+      </c>
+      <c r="H18" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2417,29 +2518,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>16</v>
       </c>
-      <c r="B19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="11">
-        <v>1.8999999999998299E-2</v>
-      </c>
-      <c r="D19" s="11">
-        <v>3.0146671490131401E-2</v>
-      </c>
-      <c r="E19" s="11">
-        <v>2.6596621957277701E-3</v>
-      </c>
-      <c r="F19" s="11">
-        <v>1.02583333333333E-2</v>
-      </c>
-      <c r="G19" s="11">
-        <v>63.025199999999998</v>
-      </c>
-      <c r="H19" t="b">
+      <c r="B19" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" s="13">
+        <v>9.7999999999999907E-2</v>
+      </c>
+      <c r="D19" s="13">
+        <v>12.577002053388</v>
+      </c>
+      <c r="E19" s="13">
+        <v>2.3442622950819601E-4</v>
+      </c>
+      <c r="F19" s="13">
+        <v>7.5000000000000002E-4</v>
+      </c>
+      <c r="G19" s="14">
+        <v>0.7792</v>
+      </c>
+      <c r="H19" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2447,30 +2548,34 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K19" s="17"/>
+      <c r="L19" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>17</v>
       </c>
-      <c r="B20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="11">
-        <v>0.68800000000000205</v>
-      </c>
-      <c r="D20" s="11">
-        <v>0.55194721844273997</v>
-      </c>
-      <c r="E20" s="11">
-        <v>3.8649015271701699E-3</v>
-      </c>
-      <c r="F20" s="11">
-        <v>1.8665000000000001E-2</v>
-      </c>
-      <c r="G20" s="11">
-        <v>124.64960000000001</v>
-      </c>
-      <c r="H20" t="b">
+      <c r="B20" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="13">
+        <v>0.29800000000000099</v>
+      </c>
+      <c r="D20" s="13">
+        <v>1.3090500162533101</v>
+      </c>
+      <c r="E20" s="13">
+        <v>1.6363387978142001E-3</v>
+      </c>
+      <c r="F20" s="13">
+        <v>5.0145161290322503E-3</v>
+      </c>
+      <c r="G20" s="14">
+        <v>22.764600000000002</v>
+      </c>
+      <c r="H20" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2479,29 +2584,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>18</v>
       </c>
-      <c r="B21" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="11">
-        <v>0.86919999999997799</v>
-      </c>
-      <c r="D21" s="11">
-        <v>0.48930641434997302</v>
-      </c>
-      <c r="E21" s="11">
-        <v>6.1959016393442496E-3</v>
-      </c>
-      <c r="F21" s="11">
-        <v>1.9137903225806399E-2</v>
-      </c>
-      <c r="G21" s="11">
-        <v>177.63919999999999</v>
-      </c>
-      <c r="H21" t="b">
+      <c r="B21" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="13">
+        <v>0.59840000000001203</v>
+      </c>
+      <c r="D21" s="13">
+        <v>0.87976453361013995</v>
+      </c>
+      <c r="E21" s="13">
+        <v>2.9445522066655302E-3</v>
+      </c>
+      <c r="F21" s="13">
+        <v>9.0640327890882093E-3</v>
+      </c>
+      <c r="G21" s="14">
+        <v>68.018199999999993</v>
+      </c>
+      <c r="H21" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2510,29 +2615,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>19</v>
       </c>
-      <c r="B22" t="s">
-        <v>14</v>
-      </c>
-      <c r="C22" s="11">
-        <v>0.44939999999999702</v>
-      </c>
-      <c r="D22" s="11">
-        <v>0.19525496544586499</v>
-      </c>
-      <c r="E22" s="11">
-        <v>3.87571782716327E-3</v>
-      </c>
-      <c r="F22" s="11">
-        <v>9.2951258002494895E-3</v>
-      </c>
-      <c r="G22" s="11">
-        <v>230.16059999999999</v>
-      </c>
-      <c r="H22" t="b">
+      <c r="B22" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="13">
+        <v>1.93999999999999E-2</v>
+      </c>
+      <c r="D22" s="13">
+        <v>12.170639899623501</v>
+      </c>
+      <c r="E22" s="13">
+        <v>6.4480874316939898E-5</v>
+      </c>
+      <c r="F22" s="13">
+        <v>3.5166666666666598E-4</v>
+      </c>
+      <c r="G22" s="14">
+        <v>0.15939999999999999</v>
+      </c>
+      <c r="H22" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2541,29 +2646,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>20</v>
       </c>
-      <c r="B23" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="11">
-        <v>0.1192</v>
-      </c>
-      <c r="D23" s="11">
-        <v>37.257762033756997</v>
-      </c>
-      <c r="E23" s="11">
-        <v>2.9781420765027299E-4</v>
-      </c>
-      <c r="F23" s="11">
-        <v>9.1903225806451601E-4</v>
-      </c>
-      <c r="G23" s="11">
-        <v>0.31993333333333301</v>
-      </c>
-      <c r="H23" t="b">
+      <c r="B23" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" s="13">
+        <v>0.29159999999999903</v>
+      </c>
+      <c r="D23" s="13">
+        <v>11.0958904109588</v>
+      </c>
+      <c r="E23" s="13">
+        <v>8.9881896703684102E-4</v>
+      </c>
+      <c r="F23" s="13">
+        <v>3.9699999999999996E-3</v>
+      </c>
+      <c r="G23" s="14">
+        <v>2.6280000000000001</v>
+      </c>
+      <c r="H23" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2572,29 +2677,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>21</v>
       </c>
-      <c r="B24" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="11">
-        <v>3.68074063492063</v>
-      </c>
-      <c r="D24" s="11">
-        <v>2.8757623752578199</v>
-      </c>
-      <c r="E24" s="11">
-        <v>1.26442232630757E-2</v>
-      </c>
-      <c r="F24" s="11">
-        <v>4.0353225806451599E-2</v>
-      </c>
-      <c r="G24" s="11">
-        <v>127.99182111111099</v>
-      </c>
-      <c r="H24" t="b">
+      <c r="B24" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="13">
+        <v>0.1638</v>
+      </c>
+      <c r="D24" s="13">
+        <v>3.5714285714285698</v>
+      </c>
+      <c r="E24" s="13">
+        <v>6.9763793407368198E-4</v>
+      </c>
+      <c r="F24" s="13">
+        <v>4.05499999999999E-3</v>
+      </c>
+      <c r="G24" s="14">
+        <v>4.5864000000000003</v>
+      </c>
+      <c r="H24" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2603,29 +2708,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>22</v>
       </c>
-      <c r="B25" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="11">
-        <v>3.65354634920635</v>
-      </c>
-      <c r="D25" s="11">
-        <v>2.39610226480427</v>
-      </c>
-      <c r="E25" s="11">
-        <v>1.24046448087431E-2</v>
-      </c>
-      <c r="F25" s="11">
-        <v>4.37609677419354E-2</v>
-      </c>
-      <c r="G25" s="11">
-        <v>152.47873193362099</v>
-      </c>
-      <c r="H25" t="b">
+      <c r="B25" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="C25" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="D25" s="13">
+        <v>1.34946210440518</v>
+      </c>
+      <c r="E25" s="13">
+        <v>1.4327157882366699E-3</v>
+      </c>
+      <c r="F25" s="13">
+        <v>6.3788172043010797E-3</v>
+      </c>
+      <c r="G25" s="14">
+        <v>37.0518</v>
+      </c>
+      <c r="H25" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2634,29 +2739,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>23</v>
       </c>
-      <c r="B26" t="s">
-        <v>18</v>
-      </c>
-      <c r="C26" s="11">
-        <v>0.24415904761903501</v>
-      </c>
-      <c r="D26" s="11">
-        <v>0.14028977951769001</v>
-      </c>
-      <c r="E26" s="11">
-        <v>3.34899765797339E-3</v>
-      </c>
-      <c r="F26" s="11">
-        <v>1.02780715916049E-2</v>
-      </c>
-      <c r="G26" s="11">
-        <v>174.03908428571401</v>
-      </c>
-      <c r="H26" t="b">
+      <c r="B26" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="13">
+        <v>0.52700000000000102</v>
+      </c>
+      <c r="D26" s="13">
+        <v>0.76734013989761096</v>
+      </c>
+      <c r="E26" s="13">
+        <v>1.6042622950819599E-3</v>
+      </c>
+      <c r="F26" s="13">
+        <v>7.8316666666667003E-3</v>
+      </c>
+      <c r="G26" s="14">
+        <v>68.678799999999995</v>
+      </c>
+      <c r="H26" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2665,29 +2770,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>24</v>
       </c>
-      <c r="B27" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="11">
-        <v>1.5239018253968699</v>
-      </c>
-      <c r="D27" s="11">
-        <v>0.46660095383969702</v>
-      </c>
-      <c r="E27" s="11">
-        <v>8.7437817800286206E-3</v>
-      </c>
-      <c r="F27" s="11">
-        <v>3.0298796799498699E-2</v>
-      </c>
-      <c r="G27" s="11">
-        <v>326.59638023809498</v>
-      </c>
-      <c r="H27" t="b">
+      <c r="B27" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="13">
+        <v>0.46880000000000099</v>
+      </c>
+      <c r="D27" s="13">
+        <v>0.53481426384322595</v>
+      </c>
+      <c r="E27" s="13">
+        <v>3.0684037540672899E-3</v>
+      </c>
+      <c r="F27" s="13">
+        <v>1.38515546639919E-2</v>
+      </c>
+      <c r="G27" s="14">
+        <v>87.656599999999997</v>
+      </c>
+      <c r="H27" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2696,29 +2801,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>25</v>
       </c>
-      <c r="B28" t="s">
-        <v>20</v>
-      </c>
-      <c r="C28" s="11">
-        <v>2.5999999999999899E-3</v>
-      </c>
-      <c r="D28" s="11">
-        <v>0.90277777777777402</v>
-      </c>
-      <c r="E28" s="11">
-        <v>7.2404371584699405E-5</v>
-      </c>
-      <c r="F28" s="11">
-        <v>2.0000000000000001E-4</v>
-      </c>
-      <c r="G28" s="11">
-        <v>0.28799999999999998</v>
-      </c>
-      <c r="H28" t="b">
+      <c r="B28" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C28" s="13">
+        <v>0.93760000000000299</v>
+      </c>
+      <c r="D28" s="13">
+        <v>0.76343460892704096</v>
+      </c>
+      <c r="E28" s="13">
+        <v>3.3075235880272902E-3</v>
+      </c>
+      <c r="F28" s="13">
+        <v>1.36029411764705E-2</v>
+      </c>
+      <c r="G28" s="14">
+        <v>122.8134</v>
+      </c>
+      <c r="H28" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2727,29 +2832,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>26</v>
       </c>
-      <c r="B29" t="s">
-        <v>21</v>
-      </c>
-      <c r="C29" s="11">
-        <v>7.2433333333336195E-2</v>
-      </c>
-      <c r="D29" s="11">
-        <v>0.31745247964280598</v>
-      </c>
-      <c r="E29" s="11">
-        <v>9.54563282213994E-4</v>
-      </c>
-      <c r="F29" s="11">
-        <v>5.0399999999999898E-3</v>
-      </c>
-      <c r="G29" s="11">
-        <v>22.817063333333302</v>
-      </c>
-      <c r="H29" t="b">
+      <c r="B29" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C29" s="13">
+        <v>0.86179999999998802</v>
+      </c>
+      <c r="D29" s="13">
+        <v>0.425967719772745</v>
+      </c>
+      <c r="E29" s="13">
+        <v>4.7279254425522102E-3</v>
+      </c>
+      <c r="F29" s="13">
+        <v>1.5907018825903899E-2</v>
+      </c>
+      <c r="G29" s="14">
+        <v>202.3158</v>
+      </c>
+      <c r="H29" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2758,29 +2863,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>27</v>
       </c>
-      <c r="B30" t="s">
-        <v>22</v>
-      </c>
-      <c r="C30" s="11">
-        <v>0.134497777777767</v>
-      </c>
-      <c r="D30" s="11">
-        <v>0.25181115868908399</v>
-      </c>
-      <c r="E30" s="11">
-        <v>1.9565573770491799E-3</v>
-      </c>
-      <c r="F30" s="11">
-        <v>8.6099999999999996E-3</v>
-      </c>
-      <c r="G30" s="11">
-        <v>53.4121595238095</v>
-      </c>
-      <c r="H30" t="b">
+      <c r="B30" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" s="13">
+        <v>1.07999999999999E-2</v>
+      </c>
+      <c r="D30" s="13">
+        <v>2.6137463697966998</v>
+      </c>
+      <c r="E30" s="13">
+        <v>4.5355191256830498E-5</v>
+      </c>
+      <c r="F30" s="13">
+        <v>1.7333333333333301E-4</v>
+      </c>
+      <c r="G30" s="14">
+        <v>0.41320000000000001</v>
+      </c>
+      <c r="H30" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2789,29 +2894,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>28</v>
       </c>
-      <c r="B31" t="s">
-        <v>23</v>
-      </c>
-      <c r="C31" s="11">
-        <v>0.46880642857144</v>
-      </c>
-      <c r="D31" s="11">
-        <v>0.425567164225987</v>
-      </c>
-      <c r="E31" s="11">
-        <v>2.1420132297957899E-3</v>
-      </c>
-      <c r="F31" s="11">
-        <v>7.2000000000000597E-3</v>
-      </c>
-      <c r="G31" s="11">
-        <v>110.16038547619</v>
-      </c>
-      <c r="H31" t="b">
+      <c r="B31" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" s="13">
+        <v>4.7400000000000497E-2</v>
+      </c>
+      <c r="D31" s="13">
+        <v>1.0119267883066301</v>
+      </c>
+      <c r="E31" s="13">
+        <v>3.6147540983606601E-4</v>
+      </c>
+      <c r="F31" s="13">
+        <v>1.54999999999999E-3</v>
+      </c>
+      <c r="G31" s="14">
+        <v>4.6841333333333299</v>
+      </c>
+      <c r="H31" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2820,29 +2925,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>29</v>
       </c>
-      <c r="B32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C32" s="11">
-        <v>0.52065269841267503</v>
-      </c>
-      <c r="D32" s="11">
-        <v>0.21579164475961701</v>
-      </c>
-      <c r="E32" s="11">
-        <v>6.4740640973667196E-3</v>
-      </c>
-      <c r="F32" s="11">
-        <v>1.53586756591047E-2</v>
-      </c>
-      <c r="G32" s="11">
-        <v>241.27565225829699</v>
-      </c>
-      <c r="H32" t="b">
+      <c r="B32" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32" s="13">
+        <v>6.7000000000000101E-2</v>
+      </c>
+      <c r="D32" s="13">
+        <v>0.34428301776911502</v>
+      </c>
+      <c r="E32" s="13">
+        <v>9.89344262295082E-4</v>
+      </c>
+      <c r="F32" s="13">
+        <v>3.3333333333333301E-3</v>
+      </c>
+      <c r="G32" s="14">
+        <v>19.460733333333302</v>
+      </c>
+      <c r="H32" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2855,25 +2960,25 @@
       <c r="A33" s="4">
         <v>30</v>
       </c>
-      <c r="B33" t="s">
-        <v>25</v>
-      </c>
-      <c r="C33" s="11">
-        <v>7.1999999999999998E-3</v>
-      </c>
-      <c r="D33" s="11">
-        <v>27.906976744186</v>
-      </c>
-      <c r="E33" s="11">
-        <v>1.6393442622950801E-5</v>
-      </c>
-      <c r="F33" s="11">
-        <v>1.38333333333333E-4</v>
-      </c>
-      <c r="G33" s="11">
-        <v>2.58E-2</v>
-      </c>
-      <c r="H33" t="b">
+      <c r="B33" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="13">
+        <v>0.61400000000000399</v>
+      </c>
+      <c r="D33" s="13">
+        <v>1.1527471303355299</v>
+      </c>
+      <c r="E33" s="13">
+        <v>1.65543803983783E-3</v>
+      </c>
+      <c r="F33" s="13">
+        <v>7.4349999999999998E-3</v>
+      </c>
+      <c r="G33" s="14">
+        <v>53.264066666666601</v>
+      </c>
+      <c r="H33" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2886,25 +2991,25 @@
       <c r="A34" s="4">
         <v>31</v>
       </c>
-      <c r="B34" t="s">
-        <v>26</v>
-      </c>
-      <c r="C34" s="11">
-        <v>2.2399999999999899E-2</v>
-      </c>
-      <c r="D34" s="11">
-        <v>1.80995475113121</v>
-      </c>
-      <c r="E34" s="11">
-        <v>1.8935307597391099E-4</v>
-      </c>
-      <c r="F34" s="11">
-        <v>9.5499999999999904E-4</v>
-      </c>
-      <c r="G34" s="11">
-        <v>1.2376</v>
-      </c>
-      <c r="H34" t="b">
+      <c r="B34" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="13">
+        <v>9.1799999999985005E-2</v>
+      </c>
+      <c r="D34" s="13">
+        <v>0.170463196909104</v>
+      </c>
+      <c r="E34" s="13">
+        <v>2.2864216463951998E-3</v>
+      </c>
+      <c r="F34" s="13">
+        <v>1.005E-2</v>
+      </c>
+      <c r="G34" s="14">
+        <v>53.853266666666599</v>
+      </c>
+      <c r="H34" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2917,25 +3022,25 @@
       <c r="A35" s="4">
         <v>32</v>
       </c>
-      <c r="B35" t="s">
-        <v>27</v>
-      </c>
-      <c r="C35" s="11">
-        <v>0.103799999999999</v>
-      </c>
-      <c r="D35" s="11">
-        <v>1.83775362062249</v>
-      </c>
-      <c r="E35" s="11">
-        <v>5.6010928961748596E-4</v>
-      </c>
-      <c r="F35" s="11">
-        <v>1.38322947214076E-3</v>
-      </c>
-      <c r="G35" s="11">
-        <v>5.6482000000000001</v>
-      </c>
-      <c r="H35" t="b">
+      <c r="B35" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="13">
+        <v>0.33222666666667</v>
+      </c>
+      <c r="D35" s="13">
+        <v>0.38132982032880602</v>
+      </c>
+      <c r="E35" s="13">
+        <v>2.4495129484438001E-3</v>
+      </c>
+      <c r="F35" s="13">
+        <v>8.1496461071789393E-3</v>
+      </c>
+      <c r="G35" s="14">
+        <v>87.123180238095202</v>
+      </c>
+      <c r="H35" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2948,25 +3053,25 @@
       <c r="A36" s="4">
         <v>33</v>
       </c>
-      <c r="B36" t="s">
-        <v>28</v>
-      </c>
-      <c r="C36" s="11">
-        <v>0.43720000000000397</v>
-      </c>
-      <c r="D36" s="11">
-        <v>0.445927696883406</v>
-      </c>
-      <c r="E36" s="11">
-        <v>2.6734972677595601E-3</v>
-      </c>
-      <c r="F36" s="11">
-        <v>5.8454728739002898E-3</v>
-      </c>
-      <c r="G36" s="11">
-        <v>98.0428</v>
-      </c>
-      <c r="H36" t="b">
+      <c r="B36" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" s="13">
+        <v>0.94603166666666905</v>
+      </c>
+      <c r="D36" s="13">
+        <v>0.98245718857136299</v>
+      </c>
+      <c r="E36" s="13">
+        <v>2.3826473488076701E-3</v>
+      </c>
+      <c r="F36" s="13">
+        <v>9.5786612300372796E-3</v>
+      </c>
+      <c r="G36" s="14">
+        <v>96.2924061904762</v>
+      </c>
+      <c r="H36" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2979,25 +3084,25 @@
       <c r="A37" s="4">
         <v>34</v>
       </c>
-      <c r="B37" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" s="11">
-        <v>4.7399999999981901E-2</v>
-      </c>
-      <c r="D37" s="11">
-        <v>2.8789527900321299E-2</v>
-      </c>
-      <c r="E37" s="11">
-        <v>3.72685764490094E-3</v>
-      </c>
-      <c r="F37" s="11">
-        <v>1.10230042750944E-2</v>
-      </c>
-      <c r="G37" s="11">
-        <v>164.64320000000001</v>
-      </c>
-      <c r="H37" t="b">
+      <c r="B37" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C37" s="13">
+        <v>2.5457857142867999E-2</v>
+      </c>
+      <c r="D37" s="13">
+        <v>1.8492558662752699E-2</v>
+      </c>
+      <c r="E37" s="13">
+        <v>2.8569606841097198E-3</v>
+      </c>
+      <c r="F37" s="13">
+        <v>9.4118676089846101E-3</v>
+      </c>
+      <c r="G37" s="14">
+        <v>137.66541238095201</v>
+      </c>
+      <c r="H37" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3010,25 +3115,25 @@
       <c r="A38" s="4">
         <v>35</v>
       </c>
-      <c r="B38" t="s">
-        <v>47</v>
-      </c>
-      <c r="C38" s="11">
-        <v>0.147242539682544</v>
-      </c>
-      <c r="D38" s="11">
-        <v>0.54289866308422996</v>
-      </c>
-      <c r="E38" s="11">
-        <v>1.4269945355191199E-3</v>
-      </c>
-      <c r="F38" s="11">
-        <v>5.3933333333333099E-3</v>
-      </c>
-      <c r="G38" s="11">
-        <v>27.1215513492063</v>
-      </c>
-      <c r="H38" t="b">
+      <c r="B38" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" s="13">
+        <v>0</v>
+      </c>
+      <c r="D38" s="13">
+        <v>0</v>
+      </c>
+      <c r="E38" s="13">
+        <v>0</v>
+      </c>
+      <c r="F38" s="13">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14">
+        <v>0</v>
+      </c>
+      <c r="H38" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3041,25 +3146,25 @@
       <c r="A39" s="4">
         <v>36</v>
       </c>
-      <c r="B39" t="s">
-        <v>48</v>
-      </c>
-      <c r="C39" s="11">
-        <v>0.84470572150072998</v>
-      </c>
-      <c r="D39" s="11">
-        <v>1.2335575212227201</v>
-      </c>
-      <c r="E39" s="11">
-        <v>1.25792349726775E-3</v>
-      </c>
-      <c r="F39" s="11">
-        <v>4.38166666666667E-3</v>
-      </c>
-      <c r="G39" s="11">
-        <v>68.477205721500695</v>
-      </c>
-      <c r="H39" t="b">
+      <c r="B39" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="13">
+        <v>7.5600000000000001E-2</v>
+      </c>
+      <c r="D39" s="13">
+        <v>13.705583756345099</v>
+      </c>
+      <c r="E39" s="13">
+        <v>1.15300546448087E-4</v>
+      </c>
+      <c r="F39" s="13">
+        <v>4.4999999999999999E-4</v>
+      </c>
+      <c r="G39" s="14">
+        <v>0.55159999999999998</v>
+      </c>
+      <c r="H39" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3072,25 +3177,25 @@
       <c r="A40" s="4">
         <v>37</v>
       </c>
-      <c r="B40" t="s">
-        <v>49</v>
-      </c>
-      <c r="C40" s="11">
-        <v>0.43367769841270798</v>
-      </c>
-      <c r="D40" s="11">
-        <v>0.33770111807430703</v>
-      </c>
-      <c r="E40" s="11">
-        <v>3.2157812906583299E-3</v>
-      </c>
-      <c r="F40" s="11">
-        <v>8.5298387096774102E-3</v>
-      </c>
-      <c r="G40" s="11">
-        <v>128.42056931457401</v>
-      </c>
-      <c r="H40" t="b">
+      <c r="B40" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="13">
+        <v>2.6599999999999201E-2</v>
+      </c>
+      <c r="D40" s="13">
+        <v>0.56101573374950997</v>
+      </c>
+      <c r="E40" s="13">
+        <v>3.72404371584699E-4</v>
+      </c>
+      <c r="F40" s="13">
+        <v>1.5149999999999901E-3</v>
+      </c>
+      <c r="G40" s="14">
+        <v>4.7413999999999996</v>
+      </c>
+      <c r="H40" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3103,25 +3208,25 @@
       <c r="A41" s="4">
         <v>38</v>
       </c>
-      <c r="B41" t="s">
-        <v>50</v>
-      </c>
-      <c r="C41" s="11">
-        <v>1.53769746031747</v>
-      </c>
-      <c r="D41" s="11">
-        <v>0.62043702926767497</v>
-      </c>
-      <c r="E41" s="11">
-        <v>6.6776896516316199E-3</v>
-      </c>
-      <c r="F41" s="11">
-        <v>1.5109411318705201E-2</v>
-      </c>
-      <c r="G41" s="11">
-        <v>247.84101976190399</v>
-      </c>
-      <c r="H41" t="b">
+      <c r="B41" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C41" s="13">
+        <v>1.8999999999998299E-2</v>
+      </c>
+      <c r="D41" s="13">
+        <v>3.0146671490131401E-2</v>
+      </c>
+      <c r="E41" s="13">
+        <v>2.6596621957277701E-3</v>
+      </c>
+      <c r="F41" s="13">
+        <v>1.02583333333333E-2</v>
+      </c>
+      <c r="G41" s="14">
+        <v>63.025199999999998</v>
+      </c>
+      <c r="H41" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3134,25 +3239,25 @@
       <c r="A42" s="4">
         <v>39</v>
       </c>
-      <c r="B42" t="s">
-        <v>51</v>
-      </c>
-      <c r="C42" s="11">
-        <v>1.73580000000001</v>
-      </c>
-      <c r="D42" s="11">
-        <v>1.1577086199870501</v>
-      </c>
-      <c r="E42" s="11">
-        <v>3.7823240392322898E-3</v>
-      </c>
-      <c r="F42" s="11">
-        <v>9.0066599768473497E-3</v>
-      </c>
-      <c r="G42" s="11">
-        <v>149.9341</v>
-      </c>
-      <c r="H42" t="b">
+      <c r="B42" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="13">
+        <v>0.68800000000000205</v>
+      </c>
+      <c r="D42" s="13">
+        <v>0.55194721844273997</v>
+      </c>
+      <c r="E42" s="13">
+        <v>3.8649015271701699E-3</v>
+      </c>
+      <c r="F42" s="13">
+        <v>1.8665000000000001E-2</v>
+      </c>
+      <c r="G42" s="14">
+        <v>124.64960000000001</v>
+      </c>
+      <c r="H42" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3165,25 +3270,25 @@
       <c r="A43" s="4">
         <v>40</v>
       </c>
-      <c r="B43" t="s">
-        <v>52</v>
-      </c>
-      <c r="C43" s="11">
-        <v>3.1172300000000002</v>
-      </c>
-      <c r="D43" s="11">
-        <v>0.86807163718326297</v>
-      </c>
-      <c r="E43" s="11">
-        <v>9.2113651909306801E-3</v>
-      </c>
-      <c r="F43" s="11">
-        <v>2.1103198242445401E-2</v>
-      </c>
-      <c r="G43" s="11">
-        <v>359.09824333333302</v>
-      </c>
-      <c r="H43" t="b">
+      <c r="B43" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C43" s="13">
+        <v>0.86919999999997799</v>
+      </c>
+      <c r="D43" s="13">
+        <v>0.48930641434997302</v>
+      </c>
+      <c r="E43" s="13">
+        <v>6.1959016393442496E-3</v>
+      </c>
+      <c r="F43" s="13">
+        <v>1.9137903225806399E-2</v>
+      </c>
+      <c r="G43" s="14">
+        <v>177.63919999999999</v>
+      </c>
+      <c r="H43" s="12" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3196,30 +3301,30 @@
       <c r="A44" s="4">
         <v>41</v>
       </c>
-      <c r="B44" t="s">
-        <v>53</v>
-      </c>
-      <c r="C44" s="11">
-        <v>1.1099999999999901</v>
-      </c>
-      <c r="D44" s="11">
-        <v>3.5044199891755299</v>
-      </c>
-      <c r="E44" s="11">
-        <v>4.7716627634660398E-3</v>
-      </c>
-      <c r="F44" s="11">
-        <v>2.1214285714285699E-2</v>
-      </c>
-      <c r="G44" s="11">
-        <v>31.674285714285698</v>
-      </c>
-      <c r="H44" t="b">
-        <f t="shared" ref="H44:H45" si="2">AND(C44&gt;$C$1, D44&gt;$D$1)</f>
+      <c r="B44" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C44" s="13">
+        <v>0.44939999999999702</v>
+      </c>
+      <c r="D44" s="13">
+        <v>0.19525496544586499</v>
+      </c>
+      <c r="E44" s="13">
+        <v>3.87571782716327E-3</v>
+      </c>
+      <c r="F44" s="13">
+        <v>9.2951258002494895E-3</v>
+      </c>
+      <c r="G44" s="14">
+        <v>230.16059999999999</v>
+      </c>
+      <c r="H44" s="12" t="b">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I44" s="5" t="b">
-        <f t="shared" ref="I44:I45" si="3">AND(F44&gt;$F$1,E44&gt;$E$1)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -3227,30 +3332,30 @@
       <c r="A45" s="4">
         <v>42</v>
       </c>
-      <c r="B45" t="s">
-        <v>54</v>
-      </c>
-      <c r="C45" s="11">
-        <v>1.16020238095237</v>
-      </c>
-      <c r="D45" s="11">
-        <v>0.75356018218390897</v>
-      </c>
-      <c r="E45" s="11">
-        <v>6.35795898090978E-3</v>
-      </c>
-      <c r="F45" s="11">
-        <v>2.5178571428571401E-2</v>
-      </c>
-      <c r="G45" s="11">
-        <v>153.96280328798099</v>
-      </c>
-      <c r="H45" t="b">
-        <f t="shared" si="2"/>
+      <c r="B45" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" s="13">
+        <v>0.1192</v>
+      </c>
+      <c r="D45" s="13">
+        <v>37.257762033756997</v>
+      </c>
+      <c r="E45" s="13">
+        <v>2.9781420765027299E-4</v>
+      </c>
+      <c r="F45" s="13">
+        <v>9.1903225806451601E-4</v>
+      </c>
+      <c r="G45" s="14">
+        <v>0.31993333333333301</v>
+      </c>
+      <c r="H45" s="12" t="b">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I45" s="5" t="b">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -3258,81 +3363,774 @@
       <c r="A46" s="4">
         <v>43</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C46" s="13">
+        <v>3.68074063492063</v>
+      </c>
+      <c r="D46" s="13">
+        <v>2.8757623752578199</v>
+      </c>
+      <c r="E46" s="13">
+        <v>1.26442232630757E-2</v>
+      </c>
+      <c r="F46" s="13">
+        <v>4.0353225806451599E-2</v>
+      </c>
+      <c r="G46" s="14">
+        <v>127.99182111111099</v>
+      </c>
+      <c r="H46" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I46" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="4">
+        <v>44</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" s="13">
+        <v>3.65354634920635</v>
+      </c>
+      <c r="D47" s="13">
+        <v>2.39610226480427</v>
+      </c>
+      <c r="E47" s="13">
+        <v>1.24046448087431E-2</v>
+      </c>
+      <c r="F47" s="13">
+        <v>4.37609677419354E-2</v>
+      </c>
+      <c r="G47" s="14">
+        <v>152.47873193362099</v>
+      </c>
+      <c r="H47" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I47" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>45</v>
+      </c>
+      <c r="B48" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C48" s="13">
+        <v>0.24415904761903501</v>
+      </c>
+      <c r="D48" s="13">
+        <v>0.14028977951769001</v>
+      </c>
+      <c r="E48" s="13">
+        <v>3.34899765797339E-3</v>
+      </c>
+      <c r="F48" s="13">
+        <v>1.02780715916049E-2</v>
+      </c>
+      <c r="G48" s="14">
+        <v>174.03908428571401</v>
+      </c>
+      <c r="H48" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I48" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="4">
+        <v>46</v>
+      </c>
+      <c r="B49" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C49" s="13">
+        <v>1.5239018253968699</v>
+      </c>
+      <c r="D49" s="13">
+        <v>0.46660095383969702</v>
+      </c>
+      <c r="E49" s="13">
+        <v>8.7437817800286206E-3</v>
+      </c>
+      <c r="F49" s="13">
+        <v>3.0298796799498699E-2</v>
+      </c>
+      <c r="G49" s="14">
+        <v>326.59638023809498</v>
+      </c>
+      <c r="H49" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I49" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="4">
+        <v>47</v>
+      </c>
+      <c r="B50" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C50" s="13">
+        <v>2.5999999999999899E-3</v>
+      </c>
+      <c r="D50" s="13">
+        <v>0.90277777777777402</v>
+      </c>
+      <c r="E50" s="13">
+        <v>7.2404371584699405E-5</v>
+      </c>
+      <c r="F50" s="13">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="G50" s="14">
+        <v>0.28799999999999998</v>
+      </c>
+      <c r="H50" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I50" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="4">
+        <v>48</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C51" s="13">
+        <v>7.2433333333336195E-2</v>
+      </c>
+      <c r="D51" s="13">
+        <v>0.31745247964280598</v>
+      </c>
+      <c r="E51" s="13">
+        <v>9.54563282213994E-4</v>
+      </c>
+      <c r="F51" s="13">
+        <v>5.0399999999999898E-3</v>
+      </c>
+      <c r="G51" s="14">
+        <v>22.817063333333302</v>
+      </c>
+      <c r="H51" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I51" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="4">
+        <v>49</v>
+      </c>
+      <c r="B52" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C52" s="13">
+        <v>0.134497777777767</v>
+      </c>
+      <c r="D52" s="13">
+        <v>0.25181115868908399</v>
+      </c>
+      <c r="E52" s="13">
+        <v>1.9565573770491799E-3</v>
+      </c>
+      <c r="F52" s="13">
+        <v>8.6099999999999996E-3</v>
+      </c>
+      <c r="G52" s="14">
+        <v>53.4121595238095</v>
+      </c>
+      <c r="H52" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I52" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="4">
+        <v>50</v>
+      </c>
+      <c r="B53" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C53" s="13">
+        <v>0.46880642857144</v>
+      </c>
+      <c r="D53" s="13">
+        <v>0.425567164225987</v>
+      </c>
+      <c r="E53" s="13">
+        <v>2.1420132297957899E-3</v>
+      </c>
+      <c r="F53" s="13">
+        <v>7.2000000000000597E-3</v>
+      </c>
+      <c r="G53" s="14">
+        <v>110.16038547619</v>
+      </c>
+      <c r="H53" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I53" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="4">
+        <v>51</v>
+      </c>
+      <c r="B54" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C54" s="13">
+        <v>0.52065269841267503</v>
+      </c>
+      <c r="D54" s="13">
+        <v>0.21579164475961701</v>
+      </c>
+      <c r="E54" s="13">
+        <v>6.4740640973667196E-3</v>
+      </c>
+      <c r="F54" s="13">
+        <v>1.53586756591047E-2</v>
+      </c>
+      <c r="G54" s="14">
+        <v>241.27565225829699</v>
+      </c>
+      <c r="H54" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I54" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="4">
+        <v>52</v>
+      </c>
+      <c r="B55" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C55" s="13">
+        <v>7.1999999999999998E-3</v>
+      </c>
+      <c r="D55" s="13">
+        <v>27.906976744186</v>
+      </c>
+      <c r="E55" s="13">
+        <v>1.6393442622950801E-5</v>
+      </c>
+      <c r="F55" s="13">
+        <v>1.38333333333333E-4</v>
+      </c>
+      <c r="G55" s="14">
+        <v>2.58E-2</v>
+      </c>
+      <c r="H55" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I55" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="4">
+        <v>53</v>
+      </c>
+      <c r="B56" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C56" s="13">
+        <v>2.2399999999999899E-2</v>
+      </c>
+      <c r="D56" s="13">
+        <v>1.80995475113121</v>
+      </c>
+      <c r="E56" s="13">
+        <v>1.8935307597391099E-4</v>
+      </c>
+      <c r="F56" s="13">
+        <v>9.5499999999999904E-4</v>
+      </c>
+      <c r="G56" s="14">
+        <v>1.2376</v>
+      </c>
+      <c r="H56" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I56" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="4">
+        <v>54</v>
+      </c>
+      <c r="B57" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C57" s="13">
+        <v>0.103799999999999</v>
+      </c>
+      <c r="D57" s="13">
+        <v>1.83775362062249</v>
+      </c>
+      <c r="E57" s="13">
+        <v>5.6010928961748596E-4</v>
+      </c>
+      <c r="F57" s="13">
+        <v>1.38322947214076E-3</v>
+      </c>
+      <c r="G57" s="14">
+        <v>5.6482000000000001</v>
+      </c>
+      <c r="H57" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I57" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
         <v>55</v>
       </c>
-      <c r="C46" s="11">
+      <c r="B58" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C58" s="13">
+        <v>0.43720000000000397</v>
+      </c>
+      <c r="D58" s="13">
+        <v>0.445927696883406</v>
+      </c>
+      <c r="E58" s="13">
+        <v>2.6734972677595601E-3</v>
+      </c>
+      <c r="F58" s="13">
+        <v>5.8454728739002898E-3</v>
+      </c>
+      <c r="G58" s="14">
+        <v>98.0428</v>
+      </c>
+      <c r="H58" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I58" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>56</v>
+      </c>
+      <c r="B59" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C59" s="13">
+        <v>4.7399999999981901E-2</v>
+      </c>
+      <c r="D59" s="13">
+        <v>2.8789527900321299E-2</v>
+      </c>
+      <c r="E59" s="13">
+        <v>3.72685764490094E-3</v>
+      </c>
+      <c r="F59" s="13">
+        <v>1.10230042750944E-2</v>
+      </c>
+      <c r="G59" s="14">
+        <v>164.64320000000001</v>
+      </c>
+      <c r="H59" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I59" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>57</v>
+      </c>
+      <c r="B60" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C60" s="13">
+        <v>0.147242539682544</v>
+      </c>
+      <c r="D60" s="13">
+        <v>0.54289866308422996</v>
+      </c>
+      <c r="E60" s="13">
+        <v>1.4269945355191199E-3</v>
+      </c>
+      <c r="F60" s="13">
+        <v>5.3933333333333099E-3</v>
+      </c>
+      <c r="G60" s="14">
+        <v>27.1215513492063</v>
+      </c>
+      <c r="H60" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I60" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="4">
+        <v>58</v>
+      </c>
+      <c r="B61" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C61" s="13">
+        <v>0.84470572150072998</v>
+      </c>
+      <c r="D61" s="13">
+        <v>1.2335575212227201</v>
+      </c>
+      <c r="E61" s="13">
+        <v>1.25792349726775E-3</v>
+      </c>
+      <c r="F61" s="13">
+        <v>4.38166666666667E-3</v>
+      </c>
+      <c r="G61" s="14">
+        <v>68.477205721500695</v>
+      </c>
+      <c r="H61" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I61" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" s="4">
+        <v>59</v>
+      </c>
+      <c r="B62" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C62" s="13">
+        <v>0.43367769841270798</v>
+      </c>
+      <c r="D62" s="13">
+        <v>0.33770111807430703</v>
+      </c>
+      <c r="E62" s="13">
+        <v>3.2157812906583299E-3</v>
+      </c>
+      <c r="F62" s="13">
+        <v>8.5298387096774102E-3</v>
+      </c>
+      <c r="G62" s="14">
+        <v>128.42056931457401</v>
+      </c>
+      <c r="H62" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I62" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="4">
+        <v>60</v>
+      </c>
+      <c r="B63" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C63" s="13">
+        <v>1.53769746031747</v>
+      </c>
+      <c r="D63" s="13">
+        <v>0.62043702926767497</v>
+      </c>
+      <c r="E63" s="13">
+        <v>6.6776896516316199E-3</v>
+      </c>
+      <c r="F63" s="13">
+        <v>1.5109411318705201E-2</v>
+      </c>
+      <c r="G63" s="14">
+        <v>247.84101976190399</v>
+      </c>
+      <c r="H63" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I63" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="4">
+        <v>61</v>
+      </c>
+      <c r="B64" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C64" s="13">
+        <v>1.73580000000001</v>
+      </c>
+      <c r="D64" s="13">
+        <v>1.1577086199870501</v>
+      </c>
+      <c r="E64" s="13">
+        <v>3.7823240392322898E-3</v>
+      </c>
+      <c r="F64" s="13">
+        <v>9.0066599768473497E-3</v>
+      </c>
+      <c r="G64" s="14">
+        <v>149.9341</v>
+      </c>
+      <c r="H64" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I64" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="4">
+        <v>62</v>
+      </c>
+      <c r="B65" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C65" s="13">
+        <v>3.1172300000000002</v>
+      </c>
+      <c r="D65" s="13">
+        <v>0.86807163718326297</v>
+      </c>
+      <c r="E65" s="13">
+        <v>9.2113651909306801E-3</v>
+      </c>
+      <c r="F65" s="13">
+        <v>2.1103198242445401E-2</v>
+      </c>
+      <c r="G65" s="14">
+        <v>359.09824333333302</v>
+      </c>
+      <c r="H65" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I65" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="4">
+        <v>63</v>
+      </c>
+      <c r="B66" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C66" s="13">
+        <v>1.1099999999999901</v>
+      </c>
+      <c r="D66" s="13">
+        <v>3.5044199891755299</v>
+      </c>
+      <c r="E66" s="13">
+        <v>4.7716627634660398E-3</v>
+      </c>
+      <c r="F66" s="13">
+        <v>2.1214285714285699E-2</v>
+      </c>
+      <c r="G66" s="14">
+        <v>31.674285714285698</v>
+      </c>
+      <c r="H66" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I66" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A67" s="4">
+        <v>64</v>
+      </c>
+      <c r="B67" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C67" s="13">
+        <v>1.16020238095237</v>
+      </c>
+      <c r="D67" s="13">
+        <v>0.75356018218390897</v>
+      </c>
+      <c r="E67" s="13">
+        <v>6.35795898090978E-3</v>
+      </c>
+      <c r="F67" s="13">
+        <v>2.5178571428571401E-2</v>
+      </c>
+      <c r="G67" s="14">
+        <v>153.96280328798099</v>
+      </c>
+      <c r="H67" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I67" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="4">
+        <v>65</v>
+      </c>
+      <c r="B68" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C68" s="13">
         <v>1.3808928571428596</v>
       </c>
-      <c r="D46" s="11">
+      <c r="D68" s="13">
         <v>0.24054718745766893</v>
       </c>
-      <c r="E46" s="11">
+      <c r="E68" s="13">
         <v>1.515236091940266E-2</v>
       </c>
-      <c r="F46" s="11">
+      <c r="F68" s="13">
         <v>2.9826343388275351E-2</v>
       </c>
-      <c r="G46" s="11">
+      <c r="G68" s="14">
         <v>574.07851785714251</v>
       </c>
-      <c r="H46" t="b">
-        <f t="shared" ref="H46:H47" si="4">AND(C46&gt;$C$1, D46&gt;$D$1)</f>
-        <v>0</v>
-      </c>
-      <c r="I46" s="5" t="b">
-        <f t="shared" ref="I46:I47" si="5">AND(F46&gt;$F$1,E46&gt;$E$1)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="6">
-        <v>44</v>
-      </c>
-      <c r="B47" s="7" t="s">
+      <c r="H68" s="12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I68" s="5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="6">
+        <v>66</v>
+      </c>
+      <c r="B69" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C47" s="12">
+      <c r="C69" s="11">
         <v>1.5939241496598595</v>
       </c>
-      <c r="D47" s="12">
+      <c r="D69" s="11">
         <v>1.4746000767244558</v>
       </c>
-      <c r="E47" s="12">
+      <c r="E69" s="11">
         <v>8.5411336707495022E-3</v>
       </c>
-      <c r="F47" s="12">
+      <c r="F69" s="11">
         <v>3.064819508448537E-2</v>
       </c>
-      <c r="G47" s="12">
+      <c r="G69" s="15">
         <v>108.23018775510153</v>
       </c>
-      <c r="H47" s="7" t="b">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I47" s="8" t="b">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
+      <c r="H69" s="7" t="b">
+        <f t="shared" ref="H69:H70" si="2">AND(C69&gt;$C$1, D69&gt;$D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="I69" s="8" t="b">
+        <f t="shared" ref="I69:I70" si="3">AND(F69&gt;$F$1,E69&gt;$E$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" s="12"/>
+      <c r="B70" s="12"/>
+      <c r="C70" s="12"/>
+      <c r="D70" s="12"/>
+      <c r="E70" s="12"/>
+      <c r="F70" s="12"/>
+      <c r="G70" s="12"/>
+      <c r="H70" s="12"/>
+      <c r="I70" s="12"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C4:C165">
+  <conditionalFormatting sqref="C4:C187">
     <cfRule type="expression" dxfId="4" priority="4">
       <formula>C4&gt;$C$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4:D66">
+  <conditionalFormatting sqref="D4:D88">
     <cfRule type="expression" dxfId="3" priority="3">
       <formula>D4&gt;$D$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E4:E87">
+  <conditionalFormatting sqref="E4:E109">
     <cfRule type="expression" dxfId="2" priority="2">
       <formula>E4&gt;$E$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F4:F118">
+  <conditionalFormatting sqref="F4:F140">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>F4&gt;$F$1</formula>
     </cfRule>

</xml_diff>